<commit_message>
Verified StockAI runs after rename
</commit_message>
<xml_diff>
--- a/res/agent_day_record.xlsx
+++ b/res/agent_day_record.xlsx
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J951"/>
+  <dimension ref="A1:J1001"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -42280,6 +42280,2206 @@
         </is>
       </c>
     </row>
+    <row r="952">
+      <c r="A952" t="n">
+        <v>1</v>
+      </c>
+      <c r="B952" t="n">
+        <v>0</v>
+      </c>
+      <c r="C952" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D952" t="n">
+        <v>0</v>
+      </c>
+      <c r="E952" t="n">
+        <v>0</v>
+      </c>
+      <c r="F952" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G952" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H952" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I952" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J952" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="953">
+      <c r="A953" t="n">
+        <v>1</v>
+      </c>
+      <c r="B953" t="n">
+        <v>1</v>
+      </c>
+      <c r="C953" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D953" t="n">
+        <v>0</v>
+      </c>
+      <c r="E953" t="n">
+        <v>0</v>
+      </c>
+      <c r="F953" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G953" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H953" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I953" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J953" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="954">
+      <c r="A954" t="n">
+        <v>1</v>
+      </c>
+      <c r="B954" t="n">
+        <v>2</v>
+      </c>
+      <c r="C954" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D954" t="n">
+        <v>0</v>
+      </c>
+      <c r="E954" t="n">
+        <v>0</v>
+      </c>
+      <c r="F954" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G954" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H954" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I954" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J954" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="955">
+      <c r="A955" t="n">
+        <v>1</v>
+      </c>
+      <c r="B955" t="n">
+        <v>3</v>
+      </c>
+      <c r="C955" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D955" t="n">
+        <v>0</v>
+      </c>
+      <c r="E955" t="n">
+        <v>0</v>
+      </c>
+      <c r="F955" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G955" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H955" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I955" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J955" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="956">
+      <c r="A956" t="n">
+        <v>1</v>
+      </c>
+      <c r="B956" t="n">
+        <v>4</v>
+      </c>
+      <c r="C956" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D956" t="n">
+        <v>0</v>
+      </c>
+      <c r="E956" t="n">
+        <v>0</v>
+      </c>
+      <c r="F956" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G956" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H956" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I956" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J956" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="957">
+      <c r="A957" t="n">
+        <v>1</v>
+      </c>
+      <c r="B957" t="n">
+        <v>5</v>
+      </c>
+      <c r="C957" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D957" t="n">
+        <v>0</v>
+      </c>
+      <c r="E957" t="n">
+        <v>0</v>
+      </c>
+      <c r="F957" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G957" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H957" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I957" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J957" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="958">
+      <c r="A958" t="n">
+        <v>1</v>
+      </c>
+      <c r="B958" t="n">
+        <v>6</v>
+      </c>
+      <c r="C958" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D958" t="n">
+        <v>0</v>
+      </c>
+      <c r="E958" t="n">
+        <v>0</v>
+      </c>
+      <c r="F958" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G958" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H958" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I958" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J958" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="959">
+      <c r="A959" t="n">
+        <v>1</v>
+      </c>
+      <c r="B959" t="n">
+        <v>7</v>
+      </c>
+      <c r="C959" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D959" t="n">
+        <v>0</v>
+      </c>
+      <c r="E959" t="n">
+        <v>0</v>
+      </c>
+      <c r="F959" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G959" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H959" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I959" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J959" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="960">
+      <c r="A960" t="n">
+        <v>1</v>
+      </c>
+      <c r="B960" t="n">
+        <v>8</v>
+      </c>
+      <c r="C960" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D960" t="n">
+        <v>0</v>
+      </c>
+      <c r="E960" t="n">
+        <v>0</v>
+      </c>
+      <c r="F960" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G960" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H960" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I960" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J960" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="961">
+      <c r="A961" t="n">
+        <v>1</v>
+      </c>
+      <c r="B961" t="n">
+        <v>9</v>
+      </c>
+      <c r="C961" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D961" t="n">
+        <v>0</v>
+      </c>
+      <c r="E961" t="n">
+        <v>0</v>
+      </c>
+      <c r="F961" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G961" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H961" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I961" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J961" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="962">
+      <c r="A962" t="n">
+        <v>1</v>
+      </c>
+      <c r="B962" t="n">
+        <v>10</v>
+      </c>
+      <c r="C962" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D962" t="n">
+        <v>0</v>
+      </c>
+      <c r="E962" t="n">
+        <v>0</v>
+      </c>
+      <c r="F962" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G962" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H962" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I962" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J962" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="963">
+      <c r="A963" t="n">
+        <v>1</v>
+      </c>
+      <c r="B963" t="n">
+        <v>11</v>
+      </c>
+      <c r="C963" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D963" t="n">
+        <v>0</v>
+      </c>
+      <c r="E963" t="n">
+        <v>0</v>
+      </c>
+      <c r="F963" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G963" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H963" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I963" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J963" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="964">
+      <c r="A964" t="n">
+        <v>1</v>
+      </c>
+      <c r="B964" t="n">
+        <v>12</v>
+      </c>
+      <c r="C964" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D964" t="n">
+        <v>0</v>
+      </c>
+      <c r="E964" t="n">
+        <v>0</v>
+      </c>
+      <c r="F964" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G964" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H964" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I964" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J964" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="965">
+      <c r="A965" t="n">
+        <v>1</v>
+      </c>
+      <c r="B965" t="n">
+        <v>13</v>
+      </c>
+      <c r="C965" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D965" t="n">
+        <v>0</v>
+      </c>
+      <c r="E965" t="n">
+        <v>0</v>
+      </c>
+      <c r="F965" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G965" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H965" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I965" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J965" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="966">
+      <c r="A966" t="n">
+        <v>1</v>
+      </c>
+      <c r="B966" t="n">
+        <v>14</v>
+      </c>
+      <c r="C966" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D966" t="n">
+        <v>0</v>
+      </c>
+      <c r="E966" t="n">
+        <v>0</v>
+      </c>
+      <c r="F966" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G966" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H966" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I966" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J966" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="967">
+      <c r="A967" t="n">
+        <v>1</v>
+      </c>
+      <c r="B967" t="n">
+        <v>15</v>
+      </c>
+      <c r="C967" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D967" t="n">
+        <v>0</v>
+      </c>
+      <c r="E967" t="n">
+        <v>0</v>
+      </c>
+      <c r="F967" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G967" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H967" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I967" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J967" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="968">
+      <c r="A968" t="n">
+        <v>1</v>
+      </c>
+      <c r="B968" t="n">
+        <v>16</v>
+      </c>
+      <c r="C968" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D968" t="n">
+        <v>0</v>
+      </c>
+      <c r="E968" t="n">
+        <v>0</v>
+      </c>
+      <c r="F968" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G968" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H968" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I968" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J968" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="969">
+      <c r="A969" t="n">
+        <v>1</v>
+      </c>
+      <c r="B969" t="n">
+        <v>17</v>
+      </c>
+      <c r="C969" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D969" t="n">
+        <v>0</v>
+      </c>
+      <c r="E969" t="n">
+        <v>0</v>
+      </c>
+      <c r="F969" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G969" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H969" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I969" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J969" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="970">
+      <c r="A970" t="n">
+        <v>1</v>
+      </c>
+      <c r="B970" t="n">
+        <v>18</v>
+      </c>
+      <c r="C970" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D970" t="n">
+        <v>0</v>
+      </c>
+      <c r="E970" t="n">
+        <v>0</v>
+      </c>
+      <c r="F970" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G970" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H970" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I970" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J970" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="971">
+      <c r="A971" t="n">
+        <v>1</v>
+      </c>
+      <c r="B971" t="n">
+        <v>19</v>
+      </c>
+      <c r="C971" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D971" t="n">
+        <v>0</v>
+      </c>
+      <c r="E971" t="n">
+        <v>0</v>
+      </c>
+      <c r="F971" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G971" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H971" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I971" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J971" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="972">
+      <c r="A972" t="n">
+        <v>1</v>
+      </c>
+      <c r="B972" t="n">
+        <v>20</v>
+      </c>
+      <c r="C972" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D972" t="n">
+        <v>0</v>
+      </c>
+      <c r="E972" t="n">
+        <v>0</v>
+      </c>
+      <c r="F972" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G972" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H972" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I972" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J972" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="973">
+      <c r="A973" t="n">
+        <v>1</v>
+      </c>
+      <c r="B973" t="n">
+        <v>21</v>
+      </c>
+      <c r="C973" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D973" t="n">
+        <v>0</v>
+      </c>
+      <c r="E973" t="n">
+        <v>0</v>
+      </c>
+      <c r="F973" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G973" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H973" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I973" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J973" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="974">
+      <c r="A974" t="n">
+        <v>1</v>
+      </c>
+      <c r="B974" t="n">
+        <v>22</v>
+      </c>
+      <c r="C974" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D974" t="n">
+        <v>0</v>
+      </c>
+      <c r="E974" t="n">
+        <v>0</v>
+      </c>
+      <c r="F974" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G974" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H974" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I974" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J974" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="975">
+      <c r="A975" t="n">
+        <v>1</v>
+      </c>
+      <c r="B975" t="n">
+        <v>23</v>
+      </c>
+      <c r="C975" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D975" t="n">
+        <v>0</v>
+      </c>
+      <c r="E975" t="n">
+        <v>0</v>
+      </c>
+      <c r="F975" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G975" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H975" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I975" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J975" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="976">
+      <c r="A976" t="n">
+        <v>1</v>
+      </c>
+      <c r="B976" t="n">
+        <v>24</v>
+      </c>
+      <c r="C976" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D976" t="n">
+        <v>0</v>
+      </c>
+      <c r="E976" t="n">
+        <v>0</v>
+      </c>
+      <c r="F976" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G976" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H976" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I976" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J976" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="977">
+      <c r="A977" t="n">
+        <v>1</v>
+      </c>
+      <c r="B977" t="n">
+        <v>25</v>
+      </c>
+      <c r="C977" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D977" t="n">
+        <v>0</v>
+      </c>
+      <c r="E977" t="n">
+        <v>0</v>
+      </c>
+      <c r="F977" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G977" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H977" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I977" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J977" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="978">
+      <c r="A978" t="n">
+        <v>1</v>
+      </c>
+      <c r="B978" t="n">
+        <v>26</v>
+      </c>
+      <c r="C978" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D978" t="n">
+        <v>0</v>
+      </c>
+      <c r="E978" t="n">
+        <v>0</v>
+      </c>
+      <c r="F978" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G978" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H978" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I978" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J978" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="979">
+      <c r="A979" t="n">
+        <v>1</v>
+      </c>
+      <c r="B979" t="n">
+        <v>27</v>
+      </c>
+      <c r="C979" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D979" t="n">
+        <v>0</v>
+      </c>
+      <c r="E979" t="n">
+        <v>0</v>
+      </c>
+      <c r="F979" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G979" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H979" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I979" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J979" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="980">
+      <c r="A980" t="n">
+        <v>1</v>
+      </c>
+      <c r="B980" t="n">
+        <v>28</v>
+      </c>
+      <c r="C980" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D980" t="n">
+        <v>0</v>
+      </c>
+      <c r="E980" t="n">
+        <v>0</v>
+      </c>
+      <c r="F980" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G980" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H980" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I980" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J980" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="981">
+      <c r="A981" t="n">
+        <v>1</v>
+      </c>
+      <c r="B981" t="n">
+        <v>29</v>
+      </c>
+      <c r="C981" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D981" t="n">
+        <v>0</v>
+      </c>
+      <c r="E981" t="n">
+        <v>0</v>
+      </c>
+      <c r="F981" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G981" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H981" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I981" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J981" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="982">
+      <c r="A982" t="n">
+        <v>1</v>
+      </c>
+      <c r="B982" t="n">
+        <v>30</v>
+      </c>
+      <c r="C982" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D982" t="n">
+        <v>0</v>
+      </c>
+      <c r="E982" t="n">
+        <v>0</v>
+      </c>
+      <c r="F982" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G982" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H982" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I982" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J982" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="983">
+      <c r="A983" t="n">
+        <v>1</v>
+      </c>
+      <c r="B983" t="n">
+        <v>31</v>
+      </c>
+      <c r="C983" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D983" t="n">
+        <v>0</v>
+      </c>
+      <c r="E983" t="n">
+        <v>0</v>
+      </c>
+      <c r="F983" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G983" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H983" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I983" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J983" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="984">
+      <c r="A984" t="n">
+        <v>1</v>
+      </c>
+      <c r="B984" t="n">
+        <v>32</v>
+      </c>
+      <c r="C984" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D984" t="n">
+        <v>0</v>
+      </c>
+      <c r="E984" t="n">
+        <v>0</v>
+      </c>
+      <c r="F984" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G984" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H984" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I984" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J984" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="985">
+      <c r="A985" t="n">
+        <v>1</v>
+      </c>
+      <c r="B985" t="n">
+        <v>33</v>
+      </c>
+      <c r="C985" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D985" t="n">
+        <v>0</v>
+      </c>
+      <c r="E985" t="n">
+        <v>0</v>
+      </c>
+      <c r="F985" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G985" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H985" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I985" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J985" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="986">
+      <c r="A986" t="n">
+        <v>1</v>
+      </c>
+      <c r="B986" t="n">
+        <v>34</v>
+      </c>
+      <c r="C986" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D986" t="n">
+        <v>0</v>
+      </c>
+      <c r="E986" t="n">
+        <v>0</v>
+      </c>
+      <c r="F986" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G986" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H986" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I986" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J986" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="987">
+      <c r="A987" t="n">
+        <v>1</v>
+      </c>
+      <c r="B987" t="n">
+        <v>35</v>
+      </c>
+      <c r="C987" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D987" t="n">
+        <v>0</v>
+      </c>
+      <c r="E987" t="n">
+        <v>0</v>
+      </c>
+      <c r="F987" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G987" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H987" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I987" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J987" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="988">
+      <c r="A988" t="n">
+        <v>1</v>
+      </c>
+      <c r="B988" t="n">
+        <v>36</v>
+      </c>
+      <c r="C988" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D988" t="n">
+        <v>0</v>
+      </c>
+      <c r="E988" t="n">
+        <v>0</v>
+      </c>
+      <c r="F988" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G988" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H988" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I988" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J988" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="989">
+      <c r="A989" t="n">
+        <v>1</v>
+      </c>
+      <c r="B989" t="n">
+        <v>37</v>
+      </c>
+      <c r="C989" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D989" t="n">
+        <v>0</v>
+      </c>
+      <c r="E989" t="n">
+        <v>0</v>
+      </c>
+      <c r="F989" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G989" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H989" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I989" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J989" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="990">
+      <c r="A990" t="n">
+        <v>1</v>
+      </c>
+      <c r="B990" t="n">
+        <v>38</v>
+      </c>
+      <c r="C990" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D990" t="n">
+        <v>0</v>
+      </c>
+      <c r="E990" t="n">
+        <v>0</v>
+      </c>
+      <c r="F990" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G990" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H990" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I990" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J990" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="991">
+      <c r="A991" t="n">
+        <v>1</v>
+      </c>
+      <c r="B991" t="n">
+        <v>39</v>
+      </c>
+      <c r="C991" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D991" t="n">
+        <v>0</v>
+      </c>
+      <c r="E991" t="n">
+        <v>0</v>
+      </c>
+      <c r="F991" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G991" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H991" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I991" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J991" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="992">
+      <c r="A992" t="n">
+        <v>1</v>
+      </c>
+      <c r="B992" t="n">
+        <v>40</v>
+      </c>
+      <c r="C992" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D992" t="n">
+        <v>0</v>
+      </c>
+      <c r="E992" t="n">
+        <v>0</v>
+      </c>
+      <c r="F992" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G992" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H992" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I992" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J992" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="993">
+      <c r="A993" t="n">
+        <v>1</v>
+      </c>
+      <c r="B993" t="n">
+        <v>41</v>
+      </c>
+      <c r="C993" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D993" t="n">
+        <v>0</v>
+      </c>
+      <c r="E993" t="n">
+        <v>0</v>
+      </c>
+      <c r="F993" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G993" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H993" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I993" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J993" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="994">
+      <c r="A994" t="n">
+        <v>1</v>
+      </c>
+      <c r="B994" t="n">
+        <v>42</v>
+      </c>
+      <c r="C994" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D994" t="n">
+        <v>0</v>
+      </c>
+      <c r="E994" t="n">
+        <v>0</v>
+      </c>
+      <c r="F994" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G994" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H994" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I994" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J994" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="995">
+      <c r="A995" t="n">
+        <v>1</v>
+      </c>
+      <c r="B995" t="n">
+        <v>43</v>
+      </c>
+      <c r="C995" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D995" t="n">
+        <v>0</v>
+      </c>
+      <c r="E995" t="n">
+        <v>0</v>
+      </c>
+      <c r="F995" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G995" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H995" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I995" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J995" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="996">
+      <c r="A996" t="n">
+        <v>1</v>
+      </c>
+      <c r="B996" t="n">
+        <v>44</v>
+      </c>
+      <c r="C996" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D996" t="n">
+        <v>0</v>
+      </c>
+      <c r="E996" t="n">
+        <v>0</v>
+      </c>
+      <c r="F996" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G996" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H996" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I996" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J996" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="997">
+      <c r="A997" t="n">
+        <v>1</v>
+      </c>
+      <c r="B997" t="n">
+        <v>45</v>
+      </c>
+      <c r="C997" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D997" t="n">
+        <v>0</v>
+      </c>
+      <c r="E997" t="n">
+        <v>0</v>
+      </c>
+      <c r="F997" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G997" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H997" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I997" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J997" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="998">
+      <c r="A998" t="n">
+        <v>1</v>
+      </c>
+      <c r="B998" t="n">
+        <v>46</v>
+      </c>
+      <c r="C998" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D998" t="n">
+        <v>0</v>
+      </c>
+      <c r="E998" t="n">
+        <v>0</v>
+      </c>
+      <c r="F998" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G998" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H998" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I998" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J998" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="999">
+      <c r="A999" t="n">
+        <v>1</v>
+      </c>
+      <c r="B999" t="n">
+        <v>47</v>
+      </c>
+      <c r="C999" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D999" t="n">
+        <v>0</v>
+      </c>
+      <c r="E999" t="n">
+        <v>0</v>
+      </c>
+      <c r="F999" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G999" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H999" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I999" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J999" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1000">
+      <c r="A1000" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1000" t="n">
+        <v>48</v>
+      </c>
+      <c r="C1000" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D1000" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1000" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1000" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G1000" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H1000" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I1000" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J1000" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
+    <row r="1001">
+      <c r="A1001" t="n">
+        <v>1</v>
+      </c>
+      <c r="B1001" t="n">
+        <v>49</v>
+      </c>
+      <c r="C1001" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="D1001" t="n">
+        <v>0</v>
+      </c>
+      <c r="E1001" t="n">
+        <v>0</v>
+      </c>
+      <c r="F1001" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="G1001" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="H1001" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="I1001" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+      <c r="J1001" t="inlineStr">
+        <is>
+          <t>no</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>